<commit_message>
Tighten analytical claims and deterministic rebuilds
</commit_message>
<xml_diff>
--- a/05_dashboard/san_diego_ops_review.xlsx
+++ b/05_dashboard/san_diego_ops_review.xlsx
@@ -139,7 +139,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="1" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="3" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -342,6 +342,7 @@
             </rich>
           </tx>
         </title>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -412,6 +413,7 @@
           <orientation val="minMax"/>
         </scaling>
         <axPos val="l"/>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="100"/>
@@ -506,6 +508,7 @@
         </scaling>
         <axPos val="l"/>
         <majorGridlines/>
+        <numFmt formatCode="#,##0" sourceLinked="0"/>
         <majorTickMark val="none"/>
         <minorTickMark val="none"/>
         <crossAx val="10"/>
@@ -696,7 +699,7 @@
   <autoFilter ref="A5:P45"/>
   <tableColumns count="16">
     <tableColumn id="1" name="Service category"/>
-    <tableColumn id="2" name="Most common record type"/>
+    <tableColumn id="2" name="Modal case_record_type"/>
     <tableColumn id="3" name="Active records"/>
     <tableColumn id="4" name="Distinct issues"/>
     <tableColumn id="5" name="Duplicate rate %"/>
@@ -1098,9 +1101,9 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
-    <col width="11" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="13" customWidth="1" min="4" max="4"/>
+    <col width="18" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -1120,7 +1123,7 @@
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
         <is>
-          <t>Generated 2026-08-09 20:51 UTC from City of San Diego Open Data Portal extracts</t>
+          <t>Generated 2026-08-10 00:18 UTC from City of San Diego Open Data Portal extracts</t>
         </is>
       </c>
     </row>
@@ -1532,7 +1535,7 @@
     <row r="29">
       <c r="A29" s="7" t="inlineStr">
         <is>
-          <t>Referred share of resolved case records</t>
+          <t>Referred share of terminal-status records</t>
         </is>
       </c>
       <c r="B29" s="9" t="n">
@@ -1585,7 +1588,7 @@
       </c>
       <c r="D31" s="7" t="inlineStr">
         <is>
-          <t>throughput</t>
+          <t>lifecycle context</t>
         </is>
       </c>
     </row>
@@ -1605,7 +1608,7 @@
       </c>
       <c r="D32" s="7" t="inlineStr">
         <is>
-          <t>throughput</t>
+          <t>lifecycle context</t>
         </is>
       </c>
     </row>
@@ -1625,7 +1628,7 @@
       </c>
       <c r="D33" s="7" t="inlineStr">
         <is>
-          <t>throughput</t>
+          <t>lifecycle context</t>
         </is>
       </c>
     </row>
@@ -1832,7 +1835,7 @@
     <row r="1">
       <c r="A1" s="12" t="inlineStr">
         <is>
-          <t>Monthly demand and recorded closures</t>
+          <t>Monthly demand and terminal-status lifecycle context</t>
         </is>
       </c>
     </row>
@@ -2754,7 +2757,7 @@
     <row r="58">
       <c r="A58" s="5" t="inlineStr">
         <is>
-          <t>Recorded case closures by month</t>
+          <t>Terminal-status records by recorded closure month</t>
         </is>
       </c>
     </row>
@@ -2894,7 +2897,7 @@
       <c r="E63" s="8" t="n">
         <v>3</v>
       </c>
-      <c r="F63" s="8" t="n">
+      <c r="F63" s="9" t="n">
         <v>146.7999999999993</v>
       </c>
       <c r="G63" s="7" t="inlineStr">
@@ -3245,7 +3248,7 @@
       <c r="E76" s="8" t="n">
         <v>2</v>
       </c>
-      <c r="F76" s="8" t="n">
+      <c r="F76" s="9" t="n">
         <v>61.60000000000218</v>
       </c>
       <c r="G76" s="7" t="inlineStr">
@@ -3411,7 +3414,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Most common record type</t>
+          <t>Modal case_record_type</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -3529,7 +3532,7 @@
       <c r="M6" s="11" t="n">
         <v>94.7</v>
       </c>
-      <c r="N6" s="7" t="n">
+      <c r="N6" s="14" t="n">
         <v>22.35</v>
       </c>
       <c r="O6" s="7" t="n">
@@ -3565,7 +3568,7 @@
       <c r="G7" s="8" t="n">
         <v>467</v>
       </c>
-      <c r="H7" s="8" t="n">
+      <c r="H7" s="9" t="n">
         <v>1358.6</v>
       </c>
       <c r="I7" s="9" t="n">
@@ -3583,7 +3586,7 @@
       <c r="M7" s="11" t="n">
         <v>90.2</v>
       </c>
-      <c r="N7" s="7" t="n">
+      <c r="N7" s="14" t="n">
         <v>19.91</v>
       </c>
       <c r="O7" s="7" t="n">
@@ -3637,7 +3640,7 @@
       <c r="M8" s="11" t="n">
         <v>85.7</v>
       </c>
-      <c r="N8" s="7" t="n">
+      <c r="N8" s="14" t="n">
         <v>14.18</v>
       </c>
       <c r="O8" s="7" t="n">
@@ -3670,10 +3673,10 @@
       <c r="F9" s="14" t="n">
         <v>6.87</v>
       </c>
-      <c r="G9" s="8" t="n">
+      <c r="G9" s="9" t="n">
         <v>1295.5</v>
       </c>
-      <c r="H9" s="8" t="n">
+      <c r="H9" s="9" t="n">
         <v>2710.1</v>
       </c>
       <c r="I9" s="9" t="n">
@@ -3691,7 +3694,7 @@
       <c r="M9" s="11" t="n">
         <v>95.7</v>
       </c>
-      <c r="N9" s="7" t="n">
+      <c r="N9" s="14" t="n">
         <v>8.640000000000001</v>
       </c>
       <c r="O9" s="7" t="n">
@@ -3745,7 +3748,7 @@
       <c r="M10" s="11" t="n">
         <v>14.6</v>
       </c>
-      <c r="N10" s="7" t="n">
+      <c r="N10" s="14" t="n">
         <v>1.1</v>
       </c>
       <c r="O10" s="7" t="n">
@@ -3781,7 +3784,7 @@
       <c r="G11" s="8" t="n">
         <v>203</v>
       </c>
-      <c r="H11" s="8" t="n">
+      <c r="H11" s="9" t="n">
         <v>1133.1</v>
       </c>
       <c r="I11" s="9" t="n">
@@ -3799,7 +3802,7 @@
       <c r="M11" s="11" t="n">
         <v>65.3</v>
       </c>
-      <c r="N11" s="7" t="n">
+      <c r="N11" s="14" t="n">
         <v>4.25</v>
       </c>
       <c r="O11" s="7" t="n">
@@ -3853,7 +3856,7 @@
       <c r="M12" s="11" t="n">
         <v>69.2</v>
       </c>
-      <c r="N12" s="7" t="n">
+      <c r="N12" s="14" t="n">
         <v>4.22</v>
       </c>
       <c r="O12" s="7" t="n">
@@ -3889,7 +3892,7 @@
       <c r="G13" s="8" t="n">
         <v>239</v>
       </c>
-      <c r="H13" s="8" t="n">
+      <c r="H13" s="9" t="n">
         <v>818.2999999999997</v>
       </c>
       <c r="I13" s="9" t="n">
@@ -3907,7 +3910,7 @@
       <c r="M13" s="11" t="n">
         <v>69.90000000000001</v>
       </c>
-      <c r="N13" s="7" t="n">
+      <c r="N13" s="14" t="n">
         <v>3.28</v>
       </c>
       <c r="O13" s="7" t="n">
@@ -3943,7 +3946,7 @@
       <c r="G14" s="8" t="n">
         <v>874</v>
       </c>
-      <c r="H14" s="8" t="n">
+      <c r="H14" s="9" t="n">
         <v>2141</v>
       </c>
       <c r="I14" s="9" t="n">
@@ -3961,7 +3964,7 @@
       <c r="M14" s="11" t="n">
         <v>89.3</v>
       </c>
-      <c r="N14" s="7" t="n">
+      <c r="N14" s="14" t="n">
         <v>3.37</v>
       </c>
       <c r="O14" s="7" t="n">
@@ -4015,7 +4018,7 @@
       <c r="M15" s="11" t="n">
         <v>28.8</v>
       </c>
-      <c r="N15" s="7" t="n">
+      <c r="N15" s="14" t="n">
         <v>1.04</v>
       </c>
       <c r="O15" s="7" t="n">
@@ -4069,7 +4072,7 @@
       <c r="M16" s="11" t="n">
         <v>70.5</v>
       </c>
-      <c r="N16" s="7" t="n">
+      <c r="N16" s="14" t="n">
         <v>2.03</v>
       </c>
       <c r="O16" s="7" t="n">
@@ -4123,7 +4126,7 @@
       <c r="M17" s="11" t="n">
         <v>77.40000000000001</v>
       </c>
-      <c r="N17" s="7" t="n">
+      <c r="N17" s="14" t="n">
         <v>2.02</v>
       </c>
       <c r="O17" s="7" t="n">
@@ -4177,7 +4180,7 @@
       <c r="M18" s="11" t="n">
         <v>55.2</v>
       </c>
-      <c r="N18" s="7" t="n">
+      <c r="N18" s="14" t="n">
         <v>1.23</v>
       </c>
       <c r="O18" s="7" t="n">
@@ -4213,7 +4216,7 @@
       <c r="G19" s="8" t="n">
         <v>158</v>
       </c>
-      <c r="H19" s="8" t="n">
+      <c r="H19" s="9" t="n">
         <v>821.6000000000001</v>
       </c>
       <c r="I19" s="9" t="n">
@@ -4231,7 +4234,7 @@
       <c r="M19" s="11" t="n">
         <v>59.9</v>
       </c>
-      <c r="N19" s="7" t="n">
+      <c r="N19" s="14" t="n">
         <v>1.25</v>
       </c>
       <c r="O19" s="7" t="n">
@@ -4267,7 +4270,7 @@
       <c r="G20" s="8" t="n">
         <v>121</v>
       </c>
-      <c r="H20" s="8" t="n">
+      <c r="H20" s="9" t="n">
         <v>511.6000000000003</v>
       </c>
       <c r="I20" s="9" t="n">
@@ -4285,7 +4288,7 @@
       <c r="M20" s="11" t="n">
         <v>61.8</v>
       </c>
-      <c r="N20" s="7" t="n">
+      <c r="N20" s="14" t="n">
         <v>1.11</v>
       </c>
       <c r="O20" s="7" t="n">
@@ -4339,7 +4342,7 @@
       <c r="M21" s="11" t="n">
         <v>100</v>
       </c>
-      <c r="N21" s="7" t="n">
+      <c r="N21" s="14" t="n">
         <v>1.78</v>
       </c>
       <c r="O21" s="7" t="n">
@@ -4375,7 +4378,7 @@
       <c r="G22" s="8" t="n">
         <v>155</v>
       </c>
-      <c r="H22" s="8" t="n">
+      <c r="H22" s="9" t="n">
         <v>537.8000000000004</v>
       </c>
       <c r="I22" s="9" t="n">
@@ -4393,7 +4396,7 @@
       <c r="M22" s="11" t="n">
         <v>61.9</v>
       </c>
-      <c r="N22" s="7" t="n">
+      <c r="N22" s="14" t="n">
         <v>1.08</v>
       </c>
       <c r="O22" s="7" t="n">
@@ -4429,7 +4432,7 @@
       <c r="G23" s="8" t="n">
         <v>89</v>
       </c>
-      <c r="H23" s="8" t="n">
+      <c r="H23" s="9" t="n">
         <v>763.6000000000006</v>
       </c>
       <c r="I23" s="9" t="n">
@@ -4447,7 +4450,7 @@
       <c r="M23" s="11" t="n">
         <v>49.9</v>
       </c>
-      <c r="N23" s="7" t="n">
+      <c r="N23" s="14" t="n">
         <v>0.84</v>
       </c>
       <c r="O23" s="7" t="n">
@@ -4480,7 +4483,7 @@
       <c r="F24" s="14" t="n">
         <v>0.9399999999999999</v>
       </c>
-      <c r="G24" s="8" t="n">
+      <c r="G24" s="9" t="n">
         <v>41.5</v>
       </c>
       <c r="H24" s="8" t="n">
@@ -4501,7 +4504,7 @@
       <c r="M24" s="11" t="n">
         <v>41</v>
       </c>
-      <c r="N24" s="7" t="n">
+      <c r="N24" s="14" t="n">
         <v>0.51</v>
       </c>
       <c r="O24" s="7" t="n">
@@ -4555,7 +4558,7 @@
       <c r="M25" s="11" t="n">
         <v>91.40000000000001</v>
       </c>
-      <c r="N25" s="7" t="n">
+      <c r="N25" s="14" t="n">
         <v>1.09</v>
       </c>
       <c r="O25" s="7" t="n">
@@ -4588,10 +4591,10 @@
       <c r="F26" s="14" t="n">
         <v>0.87</v>
       </c>
-      <c r="G26" s="8" t="n">
+      <c r="G26" s="9" t="n">
         <v>1146.5</v>
       </c>
-      <c r="H26" s="8" t="n">
+      <c r="H26" s="9" t="n">
         <v>1453.5</v>
       </c>
       <c r="I26" s="9" t="n">
@@ -4609,7 +4612,7 @@
       <c r="M26" s="11" t="n">
         <v>100</v>
       </c>
-      <c r="N26" s="7" t="n">
+      <c r="N26" s="14" t="n">
         <v>1.14</v>
       </c>
       <c r="O26" s="7" t="n">
@@ -4645,7 +4648,7 @@
       <c r="G27" s="8" t="n">
         <v>208</v>
       </c>
-      <c r="H27" s="8" t="n">
+      <c r="H27" s="9" t="n">
         <v>1082.5</v>
       </c>
       <c r="I27" s="9" t="n">
@@ -4663,7 +4666,7 @@
       <c r="M27" s="11" t="n">
         <v>61.5</v>
       </c>
-      <c r="N27" s="7" t="n">
+      <c r="N27" s="14" t="n">
         <v>0.67</v>
       </c>
       <c r="O27" s="7" t="n">
@@ -4699,7 +4702,7 @@
       <c r="G28" s="8" t="n">
         <v>279</v>
       </c>
-      <c r="H28" s="8" t="n">
+      <c r="H28" s="9" t="n">
         <v>1079.2</v>
       </c>
       <c r="I28" s="9" t="n">
@@ -4717,7 +4720,7 @@
       <c r="M28" s="11" t="n">
         <v>73.7</v>
       </c>
-      <c r="N28" s="7" t="n">
+      <c r="N28" s="14" t="n">
         <v>0.77</v>
       </c>
       <c r="O28" s="7" t="n">
@@ -4753,7 +4756,7 @@
       <c r="G29" s="8" t="n">
         <v>149</v>
       </c>
-      <c r="H29" s="8" t="n">
+      <c r="H29" s="9" t="n">
         <v>538.5000000000003</v>
       </c>
       <c r="I29" s="9" t="n">
@@ -4771,7 +4774,7 @@
       <c r="M29" s="11" t="n">
         <v>63</v>
       </c>
-      <c r="N29" s="7" t="n">
+      <c r="N29" s="14" t="n">
         <v>0.62</v>
       </c>
       <c r="O29" s="7" t="n">
@@ -4825,7 +4828,7 @@
       <c r="M30" s="11" t="n">
         <v>3.7</v>
       </c>
-      <c r="N30" s="7" t="n">
+      <c r="N30" s="14" t="n">
         <v>0.03</v>
       </c>
       <c r="O30" s="7" t="n">
@@ -4879,7 +4882,7 @@
       <c r="M31" s="11" t="n">
         <v>4.1</v>
       </c>
-      <c r="N31" s="7" t="n">
+      <c r="N31" s="14" t="n">
         <v>0.02</v>
       </c>
       <c r="O31" s="7" t="n">
@@ -4912,10 +4915,10 @@
       <c r="F32" s="14" t="n">
         <v>0.41</v>
       </c>
-      <c r="G32" s="8" t="n">
+      <c r="G32" s="9" t="n">
         <v>35.5</v>
       </c>
-      <c r="H32" s="8" t="n">
+      <c r="H32" s="9" t="n">
         <v>171.7</v>
       </c>
       <c r="I32" s="9" t="n">
@@ -4933,7 +4936,7 @@
       <c r="M32" s="11" t="n">
         <v>26.9</v>
       </c>
-      <c r="N32" s="7" t="n">
+      <c r="N32" s="14" t="n">
         <v>0.15</v>
       </c>
       <c r="O32" s="7" t="n">
@@ -4966,10 +4969,10 @@
       <c r="F33" s="14" t="n">
         <v>0.41</v>
       </c>
-      <c r="G33" s="8" t="n">
+      <c r="G33" s="9" t="n">
         <v>133.5</v>
       </c>
-      <c r="H33" s="8" t="n">
+      <c r="H33" s="9" t="n">
         <v>1257.1</v>
       </c>
       <c r="I33" s="9" t="n">
@@ -4987,7 +4990,7 @@
       <c r="M33" s="11" t="n">
         <v>52.1</v>
       </c>
-      <c r="N33" s="7" t="n">
+      <c r="N33" s="14" t="n">
         <v>0.28</v>
       </c>
       <c r="O33" s="7" t="n">
@@ -5023,7 +5026,7 @@
       <c r="G34" s="8" t="n">
         <v>34</v>
       </c>
-      <c r="H34" s="8" t="n">
+      <c r="H34" s="9" t="n">
         <v>766.3000000000002</v>
       </c>
       <c r="I34" s="9" t="n">
@@ -5041,7 +5044,7 @@
       <c r="M34" s="11" t="n">
         <v>42.6</v>
       </c>
-      <c r="N34" s="7" t="n">
+      <c r="N34" s="14" t="n">
         <v>0.17</v>
       </c>
       <c r="O34" s="7" t="n">
@@ -5077,7 +5080,7 @@
       <c r="G35" s="8" t="n">
         <v>92</v>
       </c>
-      <c r="H35" s="8" t="n">
+      <c r="H35" s="9" t="n">
         <v>523.7</v>
       </c>
       <c r="I35" s="9" t="n">
@@ -5095,7 +5098,7 @@
       <c r="M35" s="11" t="n">
         <v>52.2</v>
       </c>
-      <c r="N35" s="7" t="n">
+      <c r="N35" s="14" t="n">
         <v>0.2</v>
       </c>
       <c r="O35" s="7" t="n">
@@ -5131,7 +5134,7 @@
       <c r="G36" s="8" t="n">
         <v>193</v>
       </c>
-      <c r="H36" s="8" t="n">
+      <c r="H36" s="9" t="n">
         <v>2304.1</v>
       </c>
       <c r="I36" s="9" t="n">
@@ -5149,7 +5152,7 @@
       <c r="M36" s="11" t="n">
         <v>72.59999999999999</v>
       </c>
-      <c r="N36" s="7" t="n">
+      <c r="N36" s="14" t="n">
         <v>0.25</v>
       </c>
       <c r="O36" s="7" t="n">
@@ -5185,7 +5188,7 @@
       <c r="G37" s="8" t="n">
         <v>69</v>
       </c>
-      <c r="H37" s="8" t="n">
+      <c r="H37" s="9" t="n">
         <v>145.7</v>
       </c>
       <c r="I37" s="9" t="n">
@@ -5203,7 +5206,7 @@
       <c r="M37" s="11" t="n">
         <v>32.5</v>
       </c>
-      <c r="N37" s="7" t="n">
+      <c r="N37" s="14" t="n">
         <v>0.08</v>
       </c>
       <c r="O37" s="7" t="n">
@@ -5239,7 +5242,7 @@
       <c r="G38" s="8" t="n">
         <v>35</v>
       </c>
-      <c r="H38" s="8" t="n">
+      <c r="H38" s="9" t="n">
         <v>447.3000000000001</v>
       </c>
       <c r="I38" s="9" t="n">
@@ -5257,7 +5260,7 @@
       <c r="M38" s="11" t="n">
         <v>25</v>
       </c>
-      <c r="N38" s="7" t="n">
+      <c r="N38" s="14" t="n">
         <v>0.05</v>
       </c>
       <c r="O38" s="7" t="n">
@@ -5290,7 +5293,7 @@
       <c r="F39" s="14" t="n">
         <v>0.11</v>
       </c>
-      <c r="G39" s="8" t="n">
+      <c r="G39" s="9" t="n">
         <v>1662.5</v>
       </c>
       <c r="H39" s="8" t="n">
@@ -5311,7 +5314,7 @@
       <c r="M39" s="11" t="n">
         <v>100</v>
       </c>
-      <c r="N39" s="7" t="n">
+      <c r="N39" s="14" t="n">
         <v>0.15</v>
       </c>
       <c r="O39" s="7" t="n">
@@ -5344,10 +5347,10 @@
       <c r="F40" s="14" t="n">
         <v>0.08</v>
       </c>
-      <c r="G40" s="8" t="n">
+      <c r="G40" s="9" t="n">
         <v>47.5</v>
       </c>
-      <c r="H40" s="8" t="n">
+      <c r="H40" s="9" t="n">
         <v>780.0000000000002</v>
       </c>
       <c r="I40" s="9" t="n">
@@ -5365,7 +5368,7 @@
       <c r="M40" s="11" t="n">
         <v>37.5</v>
       </c>
-      <c r="N40" s="7" t="n">
+      <c r="N40" s="14" t="n">
         <v>0.04</v>
       </c>
       <c r="O40" s="7" t="n">
@@ -5398,10 +5401,10 @@
       <c r="F41" s="14" t="n">
         <v>0.07000000000000001</v>
       </c>
-      <c r="G41" s="8" t="n">
+      <c r="G41" s="9" t="n">
         <v>184.5</v>
       </c>
-      <c r="H41" s="8" t="n">
+      <c r="H41" s="9" t="n">
         <v>1252.100000000001</v>
       </c>
       <c r="I41" s="9" t="n">
@@ -5419,7 +5422,7 @@
       <c r="M41" s="11" t="n">
         <v>67.2</v>
       </c>
-      <c r="N41" s="7" t="n">
+      <c r="N41" s="14" t="n">
         <v>0.06</v>
       </c>
       <c r="O41" s="7" t="n">
@@ -5473,7 +5476,7 @@
       <c r="M42" s="11" t="n">
         <v>97.2</v>
       </c>
-      <c r="N42" s="7" t="n">
+      <c r="N42" s="14" t="n">
         <v>0.06</v>
       </c>
       <c r="O42" s="7" t="n">
@@ -5527,7 +5530,7 @@
       <c r="M43" s="11" t="n">
         <v>100</v>
       </c>
-      <c r="N43" s="7" t="n">
+      <c r="N43" s="14" t="n">
         <v>0</v>
       </c>
       <c r="O43" s="7" t="n">
@@ -5581,7 +5584,7 @@
       <c r="M44" s="11" t="n">
         <v>100</v>
       </c>
-      <c r="N44" s="7" t="n">
+      <c r="N44" s="14" t="n">
         <v>0</v>
       </c>
       <c r="O44" s="7" t="n">
@@ -5635,7 +5638,7 @@
       <c r="M45" s="11" t="n">
         <v>0</v>
       </c>
-      <c r="N45" s="7" t="n">
+      <c r="N45" s="14" t="n">
         <v>0</v>
       </c>
       <c r="O45" s="7" t="n">
@@ -5794,7 +5797,7 @@
       <c r="F6" s="8" t="n">
         <v>403</v>
       </c>
-      <c r="G6" s="8" t="n">
+      <c r="G6" s="9" t="n">
         <v>1633.100000000002</v>
       </c>
       <c r="H6" s="8" t="n">
@@ -5803,7 +5806,7 @@
       <c r="I6" s="11" t="n">
         <v>77.90000000000001</v>
       </c>
-      <c r="J6" s="7" t="n">
+      <c r="J6" s="11" t="n">
         <v>23.2</v>
       </c>
       <c r="K6" s="11" t="n">
@@ -5831,7 +5834,7 @@
       <c r="F7" s="8" t="n">
         <v>399</v>
       </c>
-      <c r="G7" s="8" t="n">
+      <c r="G7" s="9" t="n">
         <v>1848.800000000001</v>
       </c>
       <c r="H7" s="8" t="n">
@@ -5840,7 +5843,7 @@
       <c r="I7" s="11" t="n">
         <v>76.40000000000001</v>
       </c>
-      <c r="J7" s="7" t="n">
+      <c r="J7" s="11" t="n">
         <v>15.2</v>
       </c>
       <c r="K7" s="11" t="n">
@@ -5877,7 +5880,7 @@
       <c r="I8" s="11" t="n">
         <v>82.59999999999999</v>
       </c>
-      <c r="J8" s="7" t="n">
+      <c r="J8" s="11" t="n">
         <v>12.9</v>
       </c>
       <c r="K8" s="11" t="n">
@@ -5905,7 +5908,7 @@
       <c r="F9" s="8" t="n">
         <v>331</v>
       </c>
-      <c r="G9" s="8" t="n">
+      <c r="G9" s="9" t="n">
         <v>1745.300000000001</v>
       </c>
       <c r="H9" s="8" t="n">
@@ -5914,7 +5917,7 @@
       <c r="I9" s="11" t="n">
         <v>73.5</v>
       </c>
-      <c r="J9" s="7" t="n">
+      <c r="J9" s="11" t="n">
         <v>11.1</v>
       </c>
       <c r="K9" s="11" t="n">
@@ -5942,7 +5945,7 @@
       <c r="F10" s="8" t="n">
         <v>324</v>
       </c>
-      <c r="G10" s="8" t="n">
+      <c r="G10" s="9" t="n">
         <v>1621.9</v>
       </c>
       <c r="H10" s="8" t="n">
@@ -5951,7 +5954,7 @@
       <c r="I10" s="11" t="n">
         <v>69.3</v>
       </c>
-      <c r="J10" s="7" t="n">
+      <c r="J10" s="11" t="n">
         <v>8.1</v>
       </c>
       <c r="K10" s="11" t="n">
@@ -5988,7 +5991,7 @@
       <c r="I11" s="11" t="n">
         <v>73.40000000000001</v>
       </c>
-      <c r="J11" s="7" t="n">
+      <c r="J11" s="11" t="n">
         <v>8</v>
       </c>
       <c r="K11" s="11" t="n">
@@ -6016,7 +6019,7 @@
       <c r="F12" s="8" t="n">
         <v>194</v>
       </c>
-      <c r="G12" s="8" t="n">
+      <c r="G12" s="9" t="n">
         <v>1313.3</v>
       </c>
       <c r="H12" s="8" t="n">
@@ -6025,7 +6028,7 @@
       <c r="I12" s="11" t="n">
         <v>62.8</v>
       </c>
-      <c r="J12" s="7" t="n">
+      <c r="J12" s="11" t="n">
         <v>6.1</v>
       </c>
       <c r="K12" s="11" t="n">
@@ -6053,7 +6056,7 @@
       <c r="F13" s="8" t="n">
         <v>529</v>
       </c>
-      <c r="G13" s="8" t="n">
+      <c r="G13" s="9" t="n">
         <v>1727.7</v>
       </c>
       <c r="H13" s="8" t="n">
@@ -6062,7 +6065,7 @@
       <c r="I13" s="11" t="n">
         <v>81.90000000000001</v>
       </c>
-      <c r="J13" s="7" t="n">
+      <c r="J13" s="11" t="n">
         <v>7.5</v>
       </c>
       <c r="K13" s="11" t="n">
@@ -6087,7 +6090,7 @@
       <c r="E14" s="15" t="n">
         <v>0.251</v>
       </c>
-      <c r="F14" s="8" t="n">
+      <c r="F14" s="9" t="n">
         <v>426.5</v>
       </c>
       <c r="G14" s="8" t="n">
@@ -6099,7 +6102,7 @@
       <c r="I14" s="11" t="n">
         <v>81</v>
       </c>
-      <c r="J14" s="7" t="n">
+      <c r="J14" s="11" t="n">
         <v>6.7</v>
       </c>
       <c r="K14" s="11" t="n">
@@ -6136,7 +6139,7 @@
       <c r="I15" s="11" t="n">
         <v>92.40000000000001</v>
       </c>
-      <c r="J15" s="7" t="n">
+      <c r="J15" s="11" t="n">
         <v>1.4</v>
       </c>
       <c r="K15" s="11" t="n">
@@ -6288,7 +6291,7 @@
       <c r="C22" s="8" t="n">
         <v>4127</v>
       </c>
-      <c r="D22" s="8" t="n">
+      <c r="D22" s="9" t="n">
         <v>426.5</v>
       </c>
       <c r="E22" s="14" t="n">
@@ -6559,7 +6562,7 @@
       </c>
       <c r="B33" s="7" t="inlineStr">
         <is>
-          <t>4</t>
+          <t>8</t>
         </is>
       </c>
       <c r="C33" s="8" t="n">
@@ -6601,7 +6604,7 @@
       <c r="E34" s="8" t="n">
         <v>381</v>
       </c>
-      <c r="F34" s="8" t="n">
+      <c r="F34" s="9" t="n">
         <v>2064.7</v>
       </c>
       <c r="G34" s="8" t="n">
@@ -6631,7 +6634,7 @@
       <c r="E35" s="8" t="n">
         <v>405</v>
       </c>
-      <c r="F35" s="8" t="n">
+      <c r="F35" s="9" t="n">
         <v>1903.2</v>
       </c>
       <c r="G35" s="8" t="n">
@@ -6721,7 +6724,7 @@
       <c r="E38" s="8" t="n">
         <v>464</v>
       </c>
-      <c r="F38" s="8" t="n">
+      <c r="F38" s="9" t="n">
         <v>1786.8</v>
       </c>
       <c r="G38" s="8" t="n">
@@ -6778,10 +6781,10 @@
       <c r="D40" s="14" t="n">
         <v>3.79</v>
       </c>
-      <c r="E40" s="8" t="n">
+      <c r="E40" s="9" t="n">
         <v>555.5</v>
       </c>
-      <c r="F40" s="8" t="n">
+      <c r="F40" s="9" t="n">
         <v>1887.700000000001</v>
       </c>
       <c r="G40" s="8" t="n">
@@ -6811,7 +6814,7 @@
       <c r="E41" s="8" t="n">
         <v>469</v>
       </c>
-      <c r="F41" s="8" t="n">
+      <c r="F41" s="9" t="n">
         <v>1884.799999999999</v>
       </c>
       <c r="G41" s="8" t="n">
@@ -6871,7 +6874,7 @@
       <c r="E43" s="8" t="n">
         <v>195</v>
       </c>
-      <c r="F43" s="8" t="n">
+      <c r="F43" s="9" t="n">
         <v>1377.5</v>
       </c>
       <c r="G43" s="8" t="n">
@@ -6931,7 +6934,7 @@
       <c r="E45" s="8" t="n">
         <v>497</v>
       </c>
-      <c r="F45" s="8" t="n">
+      <c r="F45" s="9" t="n">
         <v>2044.6</v>
       </c>
       <c r="G45" s="8" t="n">
@@ -6961,7 +6964,7 @@
       <c r="E46" s="8" t="n">
         <v>240</v>
       </c>
-      <c r="F46" s="8" t="n">
+      <c r="F46" s="9" t="n">
         <v>1646.4</v>
       </c>
       <c r="G46" s="8" t="n">
@@ -6991,7 +6994,7 @@
       <c r="E47" s="8" t="n">
         <v>234</v>
       </c>
-      <c r="F47" s="8" t="n">
+      <c r="F47" s="9" t="n">
         <v>1094.000000000001</v>
       </c>
       <c r="G47" s="8" t="n">
@@ -7108,10 +7111,10 @@
       <c r="D51" s="14" t="n">
         <v>1.78</v>
       </c>
-      <c r="E51" s="8" t="n">
+      <c r="E51" s="9" t="n">
         <v>493.5</v>
       </c>
-      <c r="F51" s="8" t="n">
+      <c r="F51" s="9" t="n">
         <v>1642.8</v>
       </c>
       <c r="G51" s="8" t="n">
@@ -7138,10 +7141,10 @@
       <c r="D52" s="14" t="n">
         <v>1.7</v>
       </c>
-      <c r="E52" s="8" t="n">
+      <c r="E52" s="9" t="n">
         <v>501.5</v>
       </c>
-      <c r="F52" s="8" t="n">
+      <c r="F52" s="9" t="n">
         <v>2243.1</v>
       </c>
       <c r="G52" s="8" t="n">
@@ -7171,7 +7174,7 @@
       <c r="E53" s="8" t="n">
         <v>470</v>
       </c>
-      <c r="F53" s="8" t="n">
+      <c r="F53" s="9" t="n">
         <v>1570.2</v>
       </c>
       <c r="G53" s="8" t="n">
@@ -7231,7 +7234,7 @@
       <c r="E55" s="8" t="n">
         <v>456</v>
       </c>
-      <c r="F55" s="8" t="n">
+      <c r="F55" s="9" t="n">
         <v>1456.8</v>
       </c>
       <c r="G55" s="8" t="n">
@@ -7261,7 +7264,7 @@
       <c r="E56" s="8" t="n">
         <v>311</v>
       </c>
-      <c r="F56" s="8" t="n">
+      <c r="F56" s="9" t="n">
         <v>1573.8</v>
       </c>
       <c r="G56" s="8" t="n">
@@ -7291,7 +7294,7 @@
       <c r="E57" s="8" t="n">
         <v>334</v>
       </c>
-      <c r="F57" s="8" t="n">
+      <c r="F57" s="9" t="n">
         <v>2002.5</v>
       </c>
       <c r="G57" s="8" t="n">
@@ -7321,7 +7324,7 @@
       <c r="E58" s="8" t="n">
         <v>505</v>
       </c>
-      <c r="F58" s="8" t="n">
+      <c r="F58" s="9" t="n">
         <v>1775.999999999999</v>
       </c>
       <c r="G58" s="8" t="n">
@@ -7348,7 +7351,7 @@
       <c r="D59" s="14" t="n">
         <v>1.27</v>
       </c>
-      <c r="E59" s="8" t="n">
+      <c r="E59" s="9" t="n">
         <v>418.5</v>
       </c>
       <c r="F59" s="8" t="n">
@@ -7411,7 +7414,7 @@
       <c r="E61" s="8" t="n">
         <v>341</v>
       </c>
-      <c r="F61" s="8" t="n">
+      <c r="F61" s="9" t="n">
         <v>1464.6</v>
       </c>
       <c r="G61" s="8" t="n">
@@ -7438,10 +7441,10 @@
       <c r="D62" s="14" t="n">
         <v>1.19</v>
       </c>
-      <c r="E62" s="8" t="n">
+      <c r="E62" s="9" t="n">
         <v>331.5</v>
       </c>
-      <c r="F62" s="8" t="n">
+      <c r="F62" s="9" t="n">
         <v>1692.2</v>
       </c>
       <c r="G62" s="8" t="n">
@@ -7471,7 +7474,7 @@
       <c r="E63" s="8" t="n">
         <v>457</v>
       </c>
-      <c r="F63" s="8" t="n">
+      <c r="F63" s="9" t="n">
         <v>1861.5</v>
       </c>
       <c r="G63" s="8" t="n">
@@ -7501,7 +7504,7 @@
       <c r="E64" s="8" t="n">
         <v>438</v>
       </c>
-      <c r="F64" s="8" t="n">
+      <c r="F64" s="9" t="n">
         <v>1769.1</v>
       </c>
       <c r="G64" s="8" t="n">
@@ -7561,7 +7564,7 @@
       <c r="E66" s="8" t="n">
         <v>411</v>
       </c>
-      <c r="F66" s="8" t="n">
+      <c r="F66" s="9" t="n">
         <v>1814.8</v>
       </c>
       <c r="G66" s="8" t="n">
@@ -7591,7 +7594,7 @@
       <c r="E67" s="8" t="n">
         <v>328</v>
       </c>
-      <c r="F67" s="8" t="n">
+      <c r="F67" s="9" t="n">
         <v>1541.4</v>
       </c>
       <c r="G67" s="8" t="n">
@@ -7648,7 +7651,7 @@
       <c r="D69" s="14" t="n">
         <v>0.85</v>
       </c>
-      <c r="E69" s="8" t="n">
+      <c r="E69" s="9" t="n">
         <v>276.5</v>
       </c>
       <c r="F69" s="8" t="n">
@@ -7681,7 +7684,7 @@
       <c r="E70" s="8" t="n">
         <v>486</v>
       </c>
-      <c r="F70" s="8" t="n">
+      <c r="F70" s="9" t="n">
         <v>1733.2</v>
       </c>
       <c r="G70" s="8" t="n">
@@ -7708,10 +7711,10 @@
       <c r="D71" s="14" t="n">
         <v>0.63</v>
       </c>
-      <c r="E71" s="8" t="n">
+      <c r="E71" s="9" t="n">
         <v>507.5</v>
       </c>
-      <c r="F71" s="8" t="n">
+      <c r="F71" s="9" t="n">
         <v>1525.6</v>
       </c>
       <c r="G71" s="8" t="n">
@@ -7738,10 +7741,10 @@
       <c r="D72" s="14" t="n">
         <v>0.5600000000000001</v>
       </c>
-      <c r="E72" s="8" t="n">
+      <c r="E72" s="9" t="n">
         <v>469.5</v>
       </c>
-      <c r="F72" s="8" t="n">
+      <c r="F72" s="9" t="n">
         <v>1434.5</v>
       </c>
       <c r="G72" s="8" t="n">
@@ -7759,7 +7762,7 @@
       </c>
       <c r="B73" s="7" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>5</t>
         </is>
       </c>
       <c r="C73" s="8" t="n">
@@ -7771,7 +7774,7 @@
       <c r="E73" s="8" t="n">
         <v>585</v>
       </c>
-      <c r="F73" s="8" t="n">
+      <c r="F73" s="9" t="n">
         <v>1873.6</v>
       </c>
       <c r="G73" s="8" t="n">
@@ -7801,7 +7804,7 @@
       <c r="E74" s="8" t="n">
         <v>551</v>
       </c>
-      <c r="F74" s="8" t="n">
+      <c r="F74" s="9" t="n">
         <v>1420.200000000001</v>
       </c>
       <c r="G74" s="8" t="n">
@@ -7861,7 +7864,7 @@
       <c r="E76" s="8" t="n">
         <v>292</v>
       </c>
-      <c r="F76" s="8" t="n">
+      <c r="F76" s="9" t="n">
         <v>1440.200000000001</v>
       </c>
       <c r="G76" s="8" t="n">
@@ -7891,7 +7894,7 @@
       <c r="E77" s="8" t="n">
         <v>279</v>
       </c>
-      <c r="F77" s="8" t="n">
+      <c r="F77" s="9" t="n">
         <v>2085</v>
       </c>
       <c r="G77" s="8" t="n">
@@ -7921,7 +7924,7 @@
       <c r="E78" s="8" t="n">
         <v>588</v>
       </c>
-      <c r="F78" s="8" t="n">
+      <c r="F78" s="9" t="n">
         <v>1709.5</v>
       </c>
       <c r="G78" s="8" t="n">
@@ -7951,7 +7954,7 @@
       <c r="E79" s="8" t="n">
         <v>417</v>
       </c>
-      <c r="F79" s="8" t="n">
+      <c r="F79" s="9" t="n">
         <v>1375.000000000001</v>
       </c>
       <c r="G79" s="8" t="n">
@@ -8402,10 +8405,10 @@
       <c r="C35" s="8" t="n">
         <v>5590</v>
       </c>
-      <c r="D35" s="8" t="n">
+      <c r="D35" s="9" t="n">
         <v>1295.5</v>
       </c>
-      <c r="E35" s="8" t="n">
+      <c r="E35" s="9" t="n">
         <v>2710.1</v>
       </c>
       <c r="F35" s="8" t="n">
@@ -8441,7 +8444,7 @@
       <c r="D36" s="8" t="n">
         <v>467</v>
       </c>
-      <c r="E36" s="8" t="n">
+      <c r="E36" s="9" t="n">
         <v>1358.6</v>
       </c>
       <c r="F36" s="8" t="n">
@@ -8513,7 +8516,7 @@
       <c r="D38" s="8" t="n">
         <v>874</v>
       </c>
-      <c r="E38" s="8" t="n">
+      <c r="E38" s="9" t="n">
         <v>2141</v>
       </c>
       <c r="F38" s="8" t="n">
@@ -8582,10 +8585,10 @@
       <c r="C40" s="8" t="n">
         <v>706</v>
       </c>
-      <c r="D40" s="8" t="n">
+      <c r="D40" s="9" t="n">
         <v>1146.5</v>
       </c>
-      <c r="E40" s="8" t="n">
+      <c r="E40" s="9" t="n">
         <v>1453.5</v>
       </c>
       <c r="F40" s="8" t="n">
@@ -8621,7 +8624,7 @@
       <c r="D41" s="8" t="n">
         <v>203</v>
       </c>
-      <c r="E41" s="8" t="n">
+      <c r="E41" s="9" t="n">
         <v>1133.1</v>
       </c>
       <c r="F41" s="8" t="n">
@@ -8657,7 +8660,7 @@
       <c r="D42" s="8" t="n">
         <v>239</v>
       </c>
-      <c r="E42" s="8" t="n">
+      <c r="E42" s="9" t="n">
         <v>818.2999999999997</v>
       </c>
       <c r="F42" s="8" t="n">
@@ -8837,7 +8840,7 @@
       <c r="D47" s="8" t="n">
         <v>279</v>
       </c>
-      <c r="E47" s="8" t="n">
+      <c r="E47" s="9" t="n">
         <v>1079.2</v>
       </c>
       <c r="F47" s="8" t="n">
@@ -8873,7 +8876,7 @@
       <c r="D48" s="8" t="n">
         <v>158</v>
       </c>
-      <c r="E48" s="8" t="n">
+      <c r="E48" s="9" t="n">
         <v>821.6000000000001</v>
       </c>
       <c r="F48" s="8" t="n">
@@ -8945,7 +8948,7 @@
       <c r="D50" s="8" t="n">
         <v>121</v>
       </c>
-      <c r="E50" s="8" t="n">
+      <c r="E50" s="9" t="n">
         <v>511.6000000000003</v>
       </c>
       <c r="F50" s="8" t="n">
@@ -8981,7 +8984,7 @@
       <c r="D51" s="8" t="n">
         <v>155</v>
       </c>
-      <c r="E51" s="8" t="n">
+      <c r="E51" s="9" t="n">
         <v>537.8000000000004</v>
       </c>
       <c r="F51" s="8" t="n">
@@ -9017,7 +9020,7 @@
       <c r="D52" s="8" t="n">
         <v>208</v>
       </c>
-      <c r="E52" s="8" t="n">
+      <c r="E52" s="9" t="n">
         <v>1082.5</v>
       </c>
       <c r="F52" s="8" t="n">
@@ -9053,7 +9056,7 @@
       <c r="D53" s="8" t="n">
         <v>149</v>
       </c>
-      <c r="E53" s="8" t="n">
+      <c r="E53" s="9" t="n">
         <v>538.5000000000003</v>
       </c>
       <c r="F53" s="8" t="n">
@@ -9106,7 +9109,7 @@
       </c>
       <c r="J54" s="7" t="inlineStr">
         <is>
-          <t>Queue turns over quickly; low investigation priority</t>
+          <t>Most active records are under 90 days; lower priority under this heuristic</t>
         </is>
       </c>
     </row>
@@ -9125,7 +9128,7 @@
       <c r="D55" s="8" t="n">
         <v>89</v>
       </c>
-      <c r="E55" s="8" t="n">
+      <c r="E55" s="9" t="n">
         <v>763.6000000000006</v>
       </c>
       <c r="F55" s="8" t="n">
@@ -9178,7 +9181,7 @@
       </c>
       <c r="J56" s="7" t="inlineStr">
         <is>
-          <t>Queue turns over quickly; low investigation priority</t>
+          <t>Most active records are under 90 days; lower priority under this heuristic</t>
         </is>
       </c>
     </row>
@@ -9194,7 +9197,7 @@
       <c r="C57" s="8" t="n">
         <v>768</v>
       </c>
-      <c r="D57" s="8" t="n">
+      <c r="D57" s="9" t="n">
         <v>41.5</v>
       </c>
       <c r="E57" s="8" t="n">
@@ -9939,7 +9942,7 @@
       <c r="F92" s="11" t="n">
         <v>94.8</v>
       </c>
-      <c r="G92" s="8" t="n">
+      <c r="G92" s="9" t="n">
         <v>1292.5</v>
       </c>
       <c r="H92" s="15" t="n">
@@ -10329,7 +10332,7 @@
       <c r="F105" s="11" t="n">
         <v>96.90000000000001</v>
       </c>
-      <c r="G105" s="8" t="n">
+      <c r="G105" s="9" t="n">
         <v>1493.5</v>
       </c>
       <c r="H105" s="15" t="n">
@@ -10749,7 +10752,7 @@
       <c r="F119" s="11" t="n">
         <v>88</v>
       </c>
-      <c r="G119" s="8" t="n">
+      <c r="G119" s="9" t="n">
         <v>469.5</v>
       </c>
       <c r="H119" s="15" t="n">
@@ -10779,7 +10782,7 @@
       <c r="F120" s="11" t="n">
         <v>86.3</v>
       </c>
-      <c r="G120" s="8" t="n">
+      <c r="G120" s="9" t="n">
         <v>326.5</v>
       </c>
       <c r="H120" s="15" t="n">
@@ -10869,7 +10872,7 @@
       <c r="F123" s="11" t="n">
         <v>56.6</v>
       </c>
-      <c r="G123" s="8" t="n">
+      <c r="G123" s="9" t="n">
         <v>136.5</v>
       </c>
       <c r="H123" s="15" t="n">
@@ -10929,7 +10932,7 @@
       <c r="F125" s="11" t="n">
         <v>67.09999999999999</v>
       </c>
-      <c r="G125" s="8" t="n">
+      <c r="G125" s="9" t="n">
         <v>137.5</v>
       </c>
       <c r="H125" s="15" t="n">
@@ -11019,7 +11022,7 @@
       <c r="F128" s="11" t="n">
         <v>59.9</v>
       </c>
-      <c r="G128" s="8" t="n">
+      <c r="G128" s="9" t="n">
         <v>117.5</v>
       </c>
       <c r="H128" s="15" t="n">
@@ -11193,7 +11196,7 @@
       </c>
       <c r="D8" s="16" t="inlineStr">
         <is>
-          <t>The field carries two different meanings. For resolved records it matches (date_closed - date_requested) in 99.88% of cases, as documented. For active records — which have no close date at all — it instead matches (extract date - date_requested) in 99.63% of cases. The dictionary describes only the first meaning.</t>
+          <t>The field carries two different meanings. For terminal-status records it matches (date_closed - date_requested) in 99.88% of cases, as documented. For active records — which have no close date at all — it instead matches (extract date - date_requested) in 99.63% of cases. The dictionary describes only the first meaning.</t>
         </is>
       </c>
       <c r="E8" s="16" t="inlineStr">
@@ -11468,7 +11471,7 @@
       </c>
       <c r="E18" s="16" t="inlineStr">
         <is>
-          <t>Active is defined as status in (New, In Process); resolved as (Closed, Referred). Unmapped origins fall into an explicit '(Unknown)' channel group.</t>
+          <t>Active is defined as status in (New, In Process); terminal status as (Closed, Referred). Unmapped origins fall into an explicit '(Unknown)' channel group.</t>
         </is>
       </c>
     </row>

</xml_diff>